<commit_message>
📊 V9.2.1 daily run 2026-05-10_08:44
</commit_message>
<xml_diff>
--- a/paper_trades/dashboard_2026-05-10.xlsx
+++ b/paper_trades/dashboard_2026-05-10.xlsx
@@ -694,13 +694,13 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>43.5</v>
+        <v>43.48</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>0.72</v>
+        <v>0.67</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.88</v>
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>141.7</v>
+        <v>142</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>3.15</v>
+        <v>3.37</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>3.59</v>
@@ -828,13 +828,13 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>27.82</v>
+        <v>27.78</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>1.87</v>
+        <v>1.72</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>3.92</v>
@@ -895,13 +895,13 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>37.84</v>
+        <v>37.64</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>1.58</v>
+        <v>1.05</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>3.79</v>
@@ -962,13 +962,13 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>25.7</v>
+        <v>25.6</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-2.1</v>
+        <v>-2.48</v>
       </c>
       <c r="O8" s="8" t="n">
         <v>0.11</v>
@@ -1029,13 +1029,13 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>10.73</v>
-      </c>
-      <c r="N9" s="7" t="n">
-        <v>0.28</v>
+        <v>10.7</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>-0</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>1.68</v>
@@ -1096,13 +1096,13 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>104.4</v>
+        <v>104.1</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-0.58</v>
+        <v>-0.87</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0.75</v>
@@ -1163,13 +1163,13 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>14.54</v>
+        <v>14.55</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>-0.68</v>
+        <v>-0.61</v>
       </c>
       <c r="O11" s="8" t="n">
         <v>0.34</v>
@@ -1230,13 +1230,13 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>71.5</v>
+        <v>71.75</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>1.22</v>
+        <v>1.57</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>1.71</v>
@@ -1297,13 +1297,13 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>185.2</v>
+        <v>183.6</v>
       </c>
       <c r="N13" s="7" t="n">
-        <v>1.5</v>
+        <v>0.62</v>
       </c>
       <c r="O13" s="8" t="n">
         <v>3.15</v>
@@ -1590,7 +1590,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-10T08:28:40</t>
+          <t>محسوب في: 2026-05-10T08:44:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-10_09:57
</commit_message>
<xml_diff>
--- a/paper_trades/dashboard_2026-05-10.xlsx
+++ b/paper_trades/dashboard_2026-05-10.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,6 +151,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,13 +697,13 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>43.48</v>
+        <v>43.64</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>0.67</v>
+        <v>1.04</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.88</v>
@@ -761,16 +764,16 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>142</v>
+        <v>143.1</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>3.37</v>
+        <v>4.17</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>3.59</v>
+        <v>4.32</v>
       </c>
       <c r="P5" s="8" t="n">
         <v>-0.2</v>
@@ -828,13 +831,13 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>27.78</v>
+        <v>28</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>1.72</v>
+        <v>2.53</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>3.92</v>
@@ -895,13 +898,13 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>37.64</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>1.05</v>
+        <v>36.94</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>-0.83</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>3.79</v>
@@ -918,7 +921,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -928,33 +931,33 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>26.25</v>
+        <v>105.01</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>24.89</v>
+        <v>99.56</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>28.16</v>
+        <v>110.66</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>29.62</v>
+        <v>115.06</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>16.26</v>
+        <v>10.01</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
@@ -962,19 +965,19 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>25.6</v>
+        <v>104.2</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-2.48</v>
+        <v>-0.77</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.11</v>
+        <v>0.75</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-2.63</v>
+        <v>-2.2</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -985,7 +988,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -995,33 +998,33 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>10.7</v>
+        <v>14.64</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>10.15</v>
+        <v>13.88</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>11.29</v>
+        <v>15.34</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>11.75</v>
+        <v>15.89</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>12.8</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1029,19 +1032,19 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="N9" s="8" t="n">
-        <v>-0</v>
+        <v>14.52</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>-0.82</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>1.68</v>
+        <v>0.34</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-0.93</v>
+        <v>-2.94</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1052,22 +1055,22 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1076,19 +1079,19 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>105.01</v>
+        <v>70.64</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>99.56</v>
+        <v>66.97</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>110.66</v>
+        <v>74.7</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>115.06</v>
+        <v>77.86</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>10.01</v>
+        <v>24.18</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1099,16 +1102,16 @@
         <v>3</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>104.1</v>
+        <v>70.2</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-0.87</v>
+        <v>-0.62</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0.75</v>
+        <v>1.78</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-2.2</v>
+        <v>-1.47</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1119,43 +1122,43 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>14.64</v>
+        <v>182.46</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>13.88</v>
+        <v>173</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>15.34</v>
+        <v>191.75</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>15.89</v>
+        <v>198.98</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>23.45</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1166,16 +1169,16 @@
         <v>3</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>14.55</v>
-      </c>
-      <c r="N11" s="9" t="n">
-        <v>-0.61</v>
+        <v>184.8</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>1.28</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>0.34</v>
+        <v>3.15</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-2.94</v>
+        <v>-0.36</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1186,63 +1189,63 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>70.64</v>
+        <v>14.05</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>66.97</v>
+        <v>13.32</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>74.7</v>
+        <v>15.09</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>77.86</v>
+        <v>15.89</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>24.18</v>
+        <v>14.88</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>71.75</v>
-      </c>
-      <c r="N12" s="7" t="n">
-        <v>1.57</v>
+        <v>14.05</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>1.71</v>
+        <v>0</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>-1.47</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1253,22 +1256,22 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1277,39 +1280,39 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>182.46</v>
+        <v>15.01</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>173</v>
+        <v>14.23</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>191.75</v>
+        <v>15.74</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>198.98</v>
+        <v>16.31</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>23.45</v>
+        <v>11.78</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>53%</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>183.6</v>
-      </c>
-      <c r="N13" s="7" t="n">
-        <v>0.62</v>
+        <v>15.01</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O13" s="8" t="n">
-        <v>3.15</v>
+        <v>0</v>
       </c>
       <c r="P13" s="8" t="n">
-        <v>-0.36</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
@@ -1331,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1430,7 +1433,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1440,122 +1443,254 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>11.92</v>
+        <v>26.25</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>11.24</v>
+        <v>25.64</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.0568</v>
+        <v>-0.0232</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0316</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>12</v>
+        <v>16.26</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>33.5</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O6" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G7" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="9" t="n">
+      <c r="J7" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M5" s="8" t="n">
+      <c r="M7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="8" t="n">
+      <c r="N7" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="O7" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="P7" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -1573,7 +1708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1581,44 +1716,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>📊 إحصاءات الأداء الإجمالي</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>محسوب في: 2026-05-10T08:44:50</t>
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>محسوب في: 2026-05-10T09:57:32</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>المقياس</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>إجمالي الصفقات</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>الصفقات النشطة</t>
         </is>
@@ -1628,86 +1763,86 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>الفائزة</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>الخاسرة</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>متوسط الربح</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>+0%</t>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>+0.28%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>متوسط الخسارة</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>-4.99%</t>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>-4.1%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Profit Factor</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n">
-        <v>0</v>
+      <c r="B12" s="18" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>إجمالي P&amp;L%</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>-9.99%</t>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>-12.03%</t>
         </is>
       </c>
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>🏆 أفضل صفقة</t>
         </is>
@@ -1716,18 +1851,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2050 (2026-05-08)</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>+-4.31%</t>
+          <t>8280 (2026-05-10)</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>+0.28%</t>
         </is>
       </c>
     </row>
     <row r="17"/>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>📉 أسوأ صفقة</t>
         </is>
@@ -1739,7 +1874,7 @@
           <t>4040 (2026-05-08)</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>-5.68%</t>
         </is>
@@ -1748,7 +1883,7 @@
     <row r="20"/>
     <row r="21"/>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>📈 الأداء حسب نوع الإشارة</t>
         </is>
@@ -1756,27 +1891,27 @@
     </row>
     <row r="23"/>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Signal Type</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D24" s="22" t="inlineStr">
+      <c r="D24" s="23" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>Avg P&amp;L</t>
         </is>
@@ -1794,12 +1929,12 @@
       <c r="C25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>-5.68%</t>
         </is>
@@ -1812,26 +1947,26 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>-4.31%</t>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>33.3%</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>-2.12%</t>
         </is>
       </c>
     </row>
     <row r="27"/>
     <row r="28"/>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>🏢 الأداء حسب القطاع</t>
         </is>
@@ -1839,27 +1974,27 @@
     </row>
     <row r="30"/>
     <row r="31">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>Signal Type</t>
         </is>
       </c>
-      <c r="B31" s="22" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C31" s="22" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
+      <c r="E31" s="23" t="inlineStr">
         <is>
           <t>Avg P&amp;L</t>
         </is>
@@ -1877,7 +2012,7 @@
       <c r="C32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D32" s="16" t="inlineStr">
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -1900,7 +2035,7 @@
       <c r="C33" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -1911,18 +2046,64 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="23" t="inlineStr">
-        <is>
-          <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
-        </is>
-      </c>
-    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>+0.28%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
     <row r="37"/>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
         </is>
@@ -1943,7 +2124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2008,53 +2189,53 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>8280</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+0.28%</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+0.28%</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+0.28%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -2073,17 +2254,99 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
           <t>-4.31%</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>-4.31%</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>-4.31%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>

</xml_diff>